<commit_message>
Added second research paper
</commit_message>
<xml_diff>
--- a/Taxonomy.xlsx
+++ b/Taxonomy.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t xml:space="preserve">Index</t>
   </si>
@@ -88,13 +88,13 @@
     <t xml:space="preserve">Ruben Opdebeeck; Mahmoud Alfadel; Akond Rahman; Yutaro Kashiwa; João F. Ferreira; Raula Gaikovina Kula; Coen De Roover</t>
   </si>
   <si>
-    <t xml:space="preserve">"Vrije Universiteit Brussel, Brussels, Belgium",
-    "University of Calgary, Calgary, Canada",
-    "Auburn University, Auburn, USA",
-    "Nara Institute of Science and Technology, Nara, Japan",
-    "INESC-ID and Faculty of Engineering, University of Porto, Porto, Portugal",
-    "The University of Osaka, Osaka, Japan",
-    "Vrije Universiteit Brussel, Brussels, Belgium"</t>
+    <t xml:space="preserve">Vrije Universiteit Brussel, Brussels, Belgium,
+    University of Calgary, Calgary, Canada,
+    "Auburn University, Auburn, USA,
+    Nara Institute of Science and Technology, Nara, Japan,
+    INESC-ID and Faculty of Engineering, University of Porto, Porto, Portugal,
+    The University of Osaka, Osaka, Japan,
+    Vrije Universiteit Brussel, Brussels, Belgium</t>
   </si>
   <si>
     <t xml:space="preserve">case study</t>
@@ -119,6 +119,37 @@
   </si>
   <si>
     <t xml:space="preserve">https://doi.org/10.1145/3793302.3793355</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Secure Framework for Continuous Compliance across Heterogeneous Policy Validation Points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024 IEEE 17th International Conference on Cloud Computing (CLOUD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Takumi Yanagawa , Vikas Agarwal† , Yuji Watanabe , Lou Degenaro , Anca Sailer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IBM Research - Tokyo, Japan,
+    IBM Research - India,
+    IBM Research - Tokyo, Japan,
+    IBM Thomas J. Watson Research Center, Yorktown Heights, US,
+    IBM Thomas J. Watson Research Center, Yorktown Heights, US</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prototype</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new idea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real-life testing features</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloud Security and Compliance, Compliance as Code, Policy as Code, Continuous Compliance, Integrity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1109/CLOUD62652.2024.00029</t>
   </si>
 </sst>
 </file>
@@ -235,7 +266,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr defaultColWidth="19.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.89"/>
@@ -353,6 +384,56 @@
         <v>30</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="100.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="Q2" r:id="rId1" display="https://doi.org/10.1145/3793302.3793355"/>

</xml_diff>

<commit_message>
twelveth and thirteenth paper
</commit_message>
<xml_diff>
--- a/Taxonomy.xlsx
+++ b/Taxonomy.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="133">
   <si>
     <t xml:space="preserve">Index</t>
   </si>
@@ -408,6 +408,56 @@
   </si>
   <si>
     <t xml:space="preserve">https://arxiv.org/abs/2605.31084</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An In-Depth Analysis of eBPF-Based System Security Tools in Cloud-Native Environments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IEEE Access</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jin Her, Jongseop Kim, Jinwoo Kim, Seungsoo Lee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incheon National University, Incheon 22012, Republic of Korea,
+    Kwangwoon University, Seoul 01897, Republic of Korea,
+    Kwangwoon University, Seoul 01897, Republic of Korea,
+    Incheon National University, Incheon 22012, Republic of Korea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comparative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source code https://github.com/gjwls/ESST-eval/tree/main Diagrams,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloud native security, eBPF-based system security tools,
+    KubeArmor, Tetragon, Tracee, Falco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ieeexplore.ieee.org/abstract/document/11146725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NetEdit: An Orchestration Platform for eBPF Network Functions at Scale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACM SIGCOMM 2024 Conference (ACM SIGCOMM ’24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> "Theophilus A. Benson", "Prashanth Kannan, Prankur Gupta,
+    Balasubramanian Madhavan, Kumar Saurabh Arora, Jie Meng,
+    Martin Lau, Abhishek Dhamija, "Rajiv Krishnamurthy,
+    Srikanth Sundaresan, Neil Spring, Ying Zhang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carnegie Mellon University, Meta, Meta, Meta, Meta, Meta,
+    Meta, Meta, Meta, Meta, Meta, Meta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eBPF, Network Management, Orchestration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://dl.acm.org/doi/10.1145/3651890.3672227</t>
   </si>
 </sst>
 </file>
@@ -524,7 +574,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr defaultColWidth="19.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.89"/>
@@ -1166,6 +1216,112 @@
         <v>118</v>
       </c>
     </row>
+    <row r="13" customFormat="false" ht="86.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="114.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="Q2" r:id="rId1" display="https://doi.org/10.1145/3793302.3793355"/>
@@ -1178,8 +1334,11 @@
     <hyperlink ref="Q9" r:id="rId8" display="https://www.researchgate.net/publication/388173617_Security_and_Compliance_in_GitOps_Best_Practices_and_Challenges"/>
     <hyperlink ref="Q10" r:id="rId9" display="https://www.ijcsejournal.org/gitops-scale-multi-cluster-kubernetes/"/>
     <hyperlink ref="Q11" r:id="rId10" display="https://ijetcsit.org/index.php/ijetcsit/article/view/715"/>
-    <hyperlink ref="K12" r:id="rId11" display="https://anonymous.4open.science/r/beeline"/>
+    <hyperlink ref="K12" r:id="rId11" display="Source code (https://anonymous.4open.science/r/beeline),   Diagrams"/>
     <hyperlink ref="Q12" r:id="rId12" display="https://arxiv.org/abs/2605.31084"/>
+    <hyperlink ref="K13" r:id="rId13" display="https://github.com/gjwls/ESST-eval/tree/main"/>
+    <hyperlink ref="Q13" r:id="rId14" display="https://ieeexplore.ieee.org/abstract/document/11146725"/>
+    <hyperlink ref="Q14" r:id="rId15" display="https://dl.acm.org/doi/10.1145/3651890.3672227"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
fix: improved the track columns and added tracks of first 3 papers
</commit_message>
<xml_diff>
--- a/Taxonomy.xlsx
+++ b/Taxonomy.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="152">
   <si>
     <t xml:space="preserve">Index</t>
   </si>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Venue type [conference,Journal,whitepaper]</t>
   </si>
   <si>
-    <t xml:space="preserve">Track</t>
+    <t xml:space="preserve">Track (Research Track / Experience Track / Tool Track / Survey Track / none)</t>
   </si>
   <si>
     <t xml:space="preserve">Author names</t>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">conference</t>
   </si>
   <si>
-    <t xml:space="preserve">Research Track (research-article)</t>
+    <t xml:space="preserve">Research Track</t>
   </si>
   <si>
     <t xml:space="preserve">Ruben Opdebeeck; Mahmoud Alfadel; Akond Rahman; Yutaro Kashiwa; João F. Ferreira; Raula Gaikovina Kula; Coen De Roover</t>
@@ -128,6 +128,9 @@
     <t xml:space="preserve">2024 IEEE 17th International Conference on Cloud Computing (CLOUD)</t>
   </si>
   <si>
+    <t xml:space="preserve">Research + tools track</t>
+  </si>
+  <si>
     <t xml:space="preserve">Takumi Yanagawa , Vikas Agarwal† , Yuji Watanabe , Lou Degenaro , Anca Sailer</t>
   </si>
   <si>
@@ -159,7 +162,7 @@
     <t xml:space="preserve">2026 IEEE International Conference on Software Analysis, Evolution and Reengineering - Companion (SANER-C)</t>
   </si>
   <si>
-    <t xml:space="preserve">none (more like survey)</t>
+    <t xml:space="preserve">survey track</t>
   </si>
   <si>
     <t xml:space="preserve">Cal Önal; Indika Kumara; Filippo Scaramuzza; Marco Tonnarelli</t>
@@ -193,7 +196,7 @@
     <t xml:space="preserve">whitepaper</t>
   </si>
   <si>
-    <t xml:space="preserve">none(comparison of tools)</t>
+    <t xml:space="preserve">Tools track</t>
   </si>
   <si>
     <t xml:space="preserve">Winner Olabiyi</t>
@@ -261,9 +264,6 @@
     <t xml:space="preserve">none(ResearchGate)</t>
   </si>
   <si>
-    <t xml:space="preserve">Research Track</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dr. Aris Thorne, Dr. Lena Voss, Prof. Kenji Sato</t>
   </si>
   <si>
@@ -292,7 +292,7 @@
     <t xml:space="preserve">International Journal of Scientific Research in Computer Science, Engineering and Information Technology (IJSRCSEIT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Continuous Verification </t>
+    <t xml:space="preserve">Experience Track </t>
   </si>
   <si>
     <t xml:space="preserve">Sandeep Kamadi</t>
@@ -364,9 +364,6 @@
   </si>
   <si>
     <t xml:space="preserve">International Journal of Emerging Trends in Computer Science and Information Technology</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Research </t>
   </si>
   <si>
     <t xml:space="preserve">Nadeem Siddiqui</t>
@@ -662,7 +659,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="1" width="19.66"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="48.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -782,22 +779,22 @@
         <v>19</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>26</v>
@@ -809,10 +806,10 @@
         <v>28</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="129.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -823,31 +820,31 @@
         <v>2026</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>26</v>
@@ -859,10 +856,10 @@
         <v>28</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -873,37 +870,37 @@
         <v>2026</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>27</v>
@@ -912,10 +909,10 @@
         <v>28</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="143.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -926,34 +923,34 @@
         <v>2026</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>26</v>
@@ -965,10 +962,10 @@
         <v>28</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="100.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -979,16 +976,16 @@
         <v>2025</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>75</v>
@@ -997,7 +994,7 @@
         <v>76</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>77</v>
@@ -1006,7 +1003,7 @@
         <v>78</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>26</v>
@@ -1038,7 +1035,7 @@
         <v>82</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>83</v>
@@ -1050,7 +1047,7 @@
         <v>85</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>77</v>
@@ -1062,7 +1059,7 @@
         <v>86</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>27</v>
@@ -1091,10 +1088,10 @@
         <v>90</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>91</v>
@@ -1147,7 +1144,7 @@
         <v>99</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>100</v>
@@ -1156,7 +1153,7 @@
         <v>101</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>77</v>
@@ -1165,10 +1162,10 @@
         <v>26</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>27</v>
@@ -1197,16 +1194,16 @@
         <v>105</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>23</v>
@@ -1218,10 +1215,10 @@
         <v>78</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>27</v>
@@ -1230,10 +1227,10 @@
         <v>28</v>
       </c>
       <c r="P11" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q11" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1244,37 +1241,37 @@
         <v>2026</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="I12" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>77</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>27</v>
@@ -1283,10 +1280,10 @@
         <v>28</v>
       </c>
       <c r="P12" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q12" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="86.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1297,34 +1294,34 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>120</v>
-      </c>
       <c r="E13" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="J13" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="L13" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>26</v>
@@ -1336,10 +1333,10 @@
         <v>28</v>
       </c>
       <c r="P13" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q13" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="Q13" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="114.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1350,25 +1347,25 @@
         <v>2024</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>106</v>
+        <v>20</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="I14" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>77</v>
@@ -1380,7 +1377,7 @@
         <v>86</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>27</v>
@@ -1389,10 +1386,10 @@
         <v>28</v>
       </c>
       <c r="P14" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q14" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="Q14" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="86.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1403,34 +1400,34 @@
         <v>2026</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="I15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>77</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>26</v>
@@ -1442,10 +1439,10 @@
         <v>28</v>
       </c>
       <c r="P15" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q15" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="72.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1456,25 +1453,25 @@
         <v>2023</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>143</v>
-      </c>
       <c r="I16" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>77</v>
@@ -1483,7 +1480,7 @@
         <v>78</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M16" s="1" t="s">
         <v>26</v>
@@ -1495,10 +1492,10 @@
         <v>28</v>
       </c>
       <c r="P16" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q16" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="Q16" s="1" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="185.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1509,31 +1506,31 @@
         <v>2026</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>147</v>
-      </c>
       <c r="E17" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="I17" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>77</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L17" s="1" t="s">
         <v>26</v>
@@ -1548,10 +1545,10 @@
         <v>28</v>
       </c>
       <c r="P17" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q17" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="Q17" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>